<commit_message>
subiendo primeras cosas de agosto
</commit_message>
<xml_diff>
--- a/2026/PICHINCHA/Agosto/PICHINCHA-Agosto.xlsx
+++ b/2026/PICHINCHA/Agosto/PICHINCHA-Agosto.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sistemax\Desktop\rc-consorcio2025\2026\PICHINCHA\Julio\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sistema\Desktop\rc-consorcio2025\2026\PICHINCHA\Agosto\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E1BABF4-6169-45D5-8FEC-4D35D9F0ADD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F5D6415-1220-432B-83E3-4CBE0F637D3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="detalle y gastos" sheetId="3" r:id="rId1"/>
@@ -18,20 +18,15 @@
     <sheet name="extraordinaria" sheetId="4" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'detalle y gastos'!$A$1:$F$44</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'detalle y gastos'!$A$1:$F$46</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'prorrateo '!$A$1:$M$10</definedName>
   </definedNames>
   <calcPr calcId="181029"/>
-  <extLst>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="81">
   <si>
     <t>UF</t>
   </si>
@@ -264,13 +259,16 @@
     <t>VTO 19/07</t>
   </si>
   <si>
-    <t>Vto. 17/08</t>
-  </si>
-  <si>
-    <t>Liquidacion mes de JULIO</t>
-  </si>
-  <si>
-    <t>JULIO</t>
+    <t>RECARGA DE MATAFUEGOS</t>
+  </si>
+  <si>
+    <t>Vto. 17/09</t>
+  </si>
+  <si>
+    <t>Liquidacion mes de AGOSTO</t>
+  </si>
+  <si>
+    <t>AGOSTO</t>
   </si>
 </sst>
 </file>
@@ -283,7 +281,7 @@
     <numFmt numFmtId="166" formatCode="_ &quot;$&quot;\ * #,##0_ ;_ &quot;$&quot;\ * \-#,##0_ ;_ &quot;$&quot;\ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="167" formatCode="_-[$$-2C0A]\ * #,##0.00_-;\-[$$-2C0A]\ * #,##0.00_-;_-[$$-2C0A]\ * &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="15" x14ac:knownFonts="1">
+  <fonts count="16" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -392,6 +390,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="10">
     <fill>
@@ -1224,7 +1229,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="163">
+  <cellXfs count="165">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1532,6 +1537,8 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="4" fontId="15" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="4" fontId="15" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -1610,9 +1617,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1650,9 +1657,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -1685,26 +1692,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -1737,26 +1727,9 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1933,23 +1906,23 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H67"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:H69"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="38" customWidth="1"/>
-    <col min="2" max="2" width="40.28515625" customWidth="1"/>
-    <col min="3" max="3" width="13.5703125" customWidth="1"/>
-    <col min="4" max="4" width="7.5703125" customWidth="1"/>
-    <col min="5" max="5" width="58.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="40.33203125" customWidth="1"/>
+    <col min="3" max="3" width="13.5546875" customWidth="1"/>
+    <col min="4" max="4" width="7.5546875" customWidth="1"/>
+    <col min="5" max="5" width="58.109375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="B1" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="B2" t="s">
         <v>18</v>
       </c>
@@ -1957,27 +1930,27 @@
         <v>56</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="B3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="B4" s="4" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" ht="8.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3"/>
       <c r="B5" s="18"/>
       <c r="C5" s="3"/>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="D6" s="21"/>
       <c r="E6" s="21"/>
       <c r="F6" s="21"/>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="19" t="s">
         <v>58</v>
       </c>
@@ -1985,13 +1958,13 @@
       <c r="C7" s="53"/>
       <c r="D7" s="53"/>
       <c r="E7" s="19" t="s">
+        <v>79</v>
+      </c>
+      <c r="F7" s="88" t="s">
         <v>78</v>
       </c>
-      <c r="F7" s="88" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="3"/>
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
@@ -1999,12 +1972,12 @@
       <c r="E8" s="3"/>
       <c r="F8" s="3"/>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10" s="17" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="20" t="s">
         <v>10</v>
       </c>
@@ -2016,7 +1989,7 @@
       </c>
       <c r="F11" s="141"/>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12" s="100"/>
       <c r="B12" s="100"/>
       <c r="C12" s="94"/>
@@ -2028,13 +2001,13 @@
         <v>-369892.16424926725</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" s="100" t="s">
         <v>64</v>
       </c>
       <c r="B13" s="100"/>
-      <c r="C13" s="94">
-        <v>0</v>
+      <c r="C13" s="163">
+        <v>126912.34</v>
       </c>
       <c r="D13" s="5"/>
       <c r="E13" s="43" t="s">
@@ -2045,41 +2018,41 @@
         <v>812868.99772096006</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A14" s="101" t="s">
         <v>72</v>
       </c>
       <c r="B14" s="100"/>
-      <c r="C14" s="94">
-        <v>25643</v>
+      <c r="C14" s="163">
+        <v>26412</v>
       </c>
       <c r="D14" s="5"/>
       <c r="E14" s="43" t="s">
         <v>20</v>
       </c>
       <c r="F14" s="97">
-        <f>-(C37)</f>
-        <v>-332283.45</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+        <f>-(C39)</f>
+        <v>-1096026.9899999998</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="101" t="s">
         <v>45</v>
       </c>
       <c r="B15" s="101"/>
-      <c r="C15" s="94">
+      <c r="C15" s="163">
         <v>119786</v>
       </c>
       <c r="D15" s="31"/>
       <c r="E15" s="98"/>
       <c r="F15" s="143"/>
     </row>
-    <row r="16" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="101" t="s">
         <v>19</v>
       </c>
       <c r="B16" s="100" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C16" s="62">
         <v>54000</v>
@@ -2091,19 +2064,20 @@
         <v>74</v>
       </c>
     </row>
-    <row r="17" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="101" t="s">
         <v>70</v>
       </c>
       <c r="B17" s="100"/>
-      <c r="C17" s="62">
-        <v>0</v>
+      <c r="C17" s="164">
+        <f>100000+93414.91</f>
+        <v>193414.91</v>
       </c>
       <c r="D17" s="5"/>
       <c r="E17" s="98"/>
       <c r="F17" s="143"/>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18" s="101" t="s">
         <v>67</v>
       </c>
@@ -2114,283 +2088,306 @@
       <c r="E18" s="43"/>
       <c r="F18" s="44"/>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19" s="101" t="s">
         <v>73</v>
       </c>
       <c r="B19" s="101"/>
-      <c r="C19" s="94">
-        <v>0</v>
-      </c>
-      <c r="D19" s="5"/>
+      <c r="C19" s="163">
+        <v>161595.54999999999</v>
+      </c>
       <c r="E19" s="43"/>
       <c r="F19" s="44"/>
     </row>
-    <row r="20" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="102"/>
-      <c r="B20" s="103"/>
-      <c r="C20" s="69">
-        <f>SUM(C12:C19)</f>
-        <v>232117.66999999998</v>
-      </c>
-      <c r="E20" s="45" t="s">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A20" s="101" t="s">
+        <v>73</v>
+      </c>
+      <c r="B20" s="101"/>
+      <c r="C20" s="163">
+        <v>162681.74</v>
+      </c>
+      <c r="D20" s="5"/>
+      <c r="E20" s="43"/>
+      <c r="F20" s="44"/>
+    </row>
+    <row r="21" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A21" s="102"/>
+      <c r="B21" s="103"/>
+      <c r="C21" s="69">
+        <f>SUM(C12:C20)</f>
+        <v>877491.21</v>
+      </c>
+      <c r="E21" s="45" t="s">
         <v>43</v>
       </c>
-      <c r="F20" s="95">
-        <f>SUM(F12:F19)</f>
-        <v>110693.3834716928</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A21" s="104" t="s">
+      <c r="F21" s="95">
+        <f>SUM(F12:F20)</f>
+        <v>-653050.15652830689</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A22" s="104" t="s">
         <v>21</v>
       </c>
-      <c r="B21" s="101"/>
-      <c r="C21" s="89"/>
-      <c r="D21" s="5"/>
-      <c r="E21" s="14"/>
-      <c r="F21" s="15"/>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A22" s="101" t="s">
-        <v>63</v>
-      </c>
-      <c r="B22" s="105"/>
-      <c r="C22" s="94">
-        <v>91370</v>
-      </c>
+      <c r="B22" s="101"/>
+      <c r="C22" s="89"/>
       <c r="D22" s="5"/>
       <c r="E22" s="14"/>
       <c r="F22" s="15"/>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23" s="101" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="B23" s="105"/>
-      <c r="C23" s="94">
-        <v>5837.2</v>
+      <c r="C23" s="163">
+        <v>182740</v>
       </c>
       <c r="D23" s="5"/>
       <c r="E23" s="14"/>
       <c r="F23" s="15"/>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24" s="101" t="s">
-        <v>75</v>
+        <v>68</v>
       </c>
       <c r="B24" s="105"/>
       <c r="C24" s="94">
-        <v>2958.58</v>
+        <v>5837.2</v>
       </c>
       <c r="D24" s="5"/>
       <c r="E24" s="14"/>
       <c r="F24" s="15"/>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A25" s="87" t="s">
-        <v>69</v>
-      </c>
-      <c r="B25" s="106"/>
-      <c r="C25" s="94">
-        <f>718194.55-332283.45</f>
-        <v>385911.10000000003</v>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A25" s="101" t="s">
+        <v>77</v>
+      </c>
+      <c r="B25" s="105"/>
+      <c r="C25" s="163">
+        <v>27000</v>
       </c>
       <c r="D25" s="5"/>
       <c r="E25" s="14"/>
       <c r="F25" s="15"/>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A26" s="23"/>
-      <c r="B26" s="24"/>
-      <c r="C26" s="99">
-        <f>SUM(C21:C25)</f>
-        <v>486076.88</v>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A26" s="101" t="s">
+        <v>75</v>
+      </c>
+      <c r="B26" s="105"/>
+      <c r="C26" s="94">
+        <v>2958.58</v>
       </c>
       <c r="D26" s="5"/>
-      <c r="E26" s="5"/>
-      <c r="F26" s="40"/>
-      <c r="G26" s="6"/>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27" s="33" t="s">
-        <v>12</v>
-      </c>
-      <c r="B27" s="34"/>
-      <c r="C27" s="35">
-        <f>+C26+C20</f>
-        <v>718194.55</v>
+      <c r="E26" s="14"/>
+      <c r="F26" s="15"/>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A27" s="87" t="s">
+        <v>69</v>
+      </c>
+      <c r="B27" s="106"/>
+      <c r="C27" s="94">
+        <f>718194.55-332283.45</f>
+        <v>385911.10000000003</v>
       </c>
       <c r="D27" s="5"/>
       <c r="E27" s="14"/>
       <c r="F27" s="15"/>
     </row>
-    <row r="28" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="54" t="s">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A28" s="23"/>
+      <c r="B28" s="24"/>
+      <c r="C28" s="99">
+        <f>SUM(C22:C27)</f>
+        <v>604446.88</v>
+      </c>
+      <c r="D28" s="5"/>
+      <c r="E28" s="5"/>
+      <c r="F28" s="40"/>
+      <c r="G28" s="6"/>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A29" s="33" t="s">
+        <v>12</v>
+      </c>
+      <c r="B29" s="34"/>
+      <c r="C29" s="35">
+        <f>+C28+C21</f>
+        <v>1481938.0899999999</v>
+      </c>
+      <c r="D29" s="5"/>
+      <c r="E29" s="14"/>
+      <c r="F29" s="15"/>
+    </row>
+    <row r="30" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="54" t="s">
         <v>24</v>
       </c>
-      <c r="B28" s="64"/>
-      <c r="C28" s="65"/>
-      <c r="E28" s="14"/>
-      <c r="F28" s="15"/>
-    </row>
-    <row r="29" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="17" t="s">
+      <c r="B30" s="64"/>
+      <c r="C30" s="65"/>
+      <c r="E30" s="14"/>
+      <c r="F30" s="15"/>
+    </row>
+    <row r="31" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="17" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="30" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="32"/>
-      <c r="B30" s="21"/>
-      <c r="C30" s="39"/>
-      <c r="F30" s="6"/>
-    </row>
-    <row r="31" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="37"/>
-      <c r="B31" s="36"/>
-      <c r="C31" s="38">
-        <v>0</v>
-      </c>
-      <c r="F31" s="6"/>
-    </row>
-    <row r="32" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="46"/>
-      <c r="B32" s="47"/>
-      <c r="C32" s="38">
-        <v>0</v>
-      </c>
+    <row r="32" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="32"/>
+      <c r="B32" s="21"/>
+      <c r="C32" s="39"/>
       <c r="F32" s="6"/>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A33" s="60"/>
-      <c r="B33" s="61"/>
-      <c r="C33" s="63"/>
+    <row r="33" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="37"/>
+      <c r="B33" s="36"/>
+      <c r="C33" s="38">
+        <v>0</v>
+      </c>
       <c r="F33" s="6"/>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A34" s="60"/>
-      <c r="B34" s="67"/>
-      <c r="C34" s="68"/>
+    <row r="34" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="46"/>
+      <c r="B34" s="47"/>
+      <c r="C34" s="38">
+        <v>0</v>
+      </c>
       <c r="F34" s="6"/>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35" s="60"/>
-      <c r="B35" s="66"/>
-      <c r="C35" s="63">
-        <v>0</v>
-      </c>
+      <c r="B35" s="61"/>
+      <c r="C35" s="63"/>
       <c r="F35" s="6"/>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A36" s="48" t="s">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A36" s="60"/>
+      <c r="B36" s="67"/>
+      <c r="C36" s="68"/>
+      <c r="F36" s="6"/>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A37" s="60"/>
+      <c r="B37" s="66"/>
+      <c r="C37" s="63">
+        <v>0</v>
+      </c>
+      <c r="F37" s="6"/>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A38" s="48" t="s">
         <v>23</v>
       </c>
-      <c r="B36" s="49"/>
-      <c r="C36" s="50">
-        <f>SUM(C31:C35)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
+      <c r="B38" s="49"/>
+      <c r="C38" s="50">
+        <f>SUM(C33:C37)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
         <v>54</v>
       </c>
-      <c r="C37" s="38">
-        <f>C27-C25</f>
-        <v>332283.45</v>
-      </c>
-      <c r="F37" s="6"/>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A38" s="5" t="s">
+      <c r="C39" s="38">
+        <f>C29-C27</f>
+        <v>1096026.9899999998</v>
+      </c>
+      <c r="F39" s="6"/>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A40" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="C38" s="59">
-        <f>+C27</f>
-        <v>718194.55</v>
-      </c>
-      <c r="F38" s="6"/>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A39" s="48" t="s">
+      <c r="C40" s="59">
+        <f>+C29</f>
+        <v>1481938.0899999999</v>
+      </c>
+      <c r="F40" s="6"/>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A41" s="48" t="s">
         <v>13</v>
       </c>
-      <c r="B39" s="49"/>
-      <c r="C39" s="50">
-        <f>+C27+C36</f>
-        <v>718194.55</v>
-      </c>
-      <c r="E39" s="11"/>
-    </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="D44" s="6"/>
-    </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="D45" s="11"/>
-      <c r="E45" s="11"/>
-    </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B46" s="142"/>
-      <c r="C46" s="142"/>
-      <c r="D46" s="142"/>
-      <c r="E46" s="142"/>
-    </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B47" s="142"/>
-      <c r="C47" s="142"/>
-      <c r="D47" s="142"/>
-      <c r="E47" s="142"/>
-    </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B41" s="49"/>
+      <c r="C41" s="50">
+        <f>+C29+C38</f>
+        <v>1481938.0899999999</v>
+      </c>
+      <c r="E41" s="11"/>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="D46" s="6"/>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="D47" s="11"/>
+      <c r="E47" s="11"/>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B48" s="142"/>
       <c r="C48" s="142"/>
       <c r="D48" s="142"/>
       <c r="E48" s="142"/>
     </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A60" s="14"/>
-      <c r="B60" s="13"/>
-      <c r="C60" s="15"/>
-    </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A61" s="13"/>
-      <c r="B61" s="13"/>
-      <c r="C61" s="13"/>
-    </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A62" s="13"/>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B49" s="142"/>
+      <c r="C49" s="142"/>
+      <c r="D49" s="142"/>
+      <c r="E49" s="142"/>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B50" s="142"/>
+      <c r="C50" s="142"/>
+      <c r="D50" s="142"/>
+      <c r="E50" s="142"/>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A62" s="14"/>
       <c r="B62" s="13"/>
-      <c r="C62" s="13"/>
-    </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C62" s="15"/>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A63" s="13"/>
       <c r="B63" s="13"/>
       <c r="C63" s="13"/>
     </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A64" s="13"/>
       <c r="B64" s="13"/>
       <c r="C64" s="13"/>
     </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A65" s="13"/>
       <c r="B65" s="13"/>
       <c r="C65" s="13"/>
     </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A66" s="13"/>
       <c r="B66" s="13"/>
       <c r="C66" s="13"/>
     </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A67" s="13"/>
       <c r="B67" s="13"/>
       <c r="C67" s="13"/>
     </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A68" s="13"/>
+      <c r="B68" s="13"/>
+      <c r="C68" s="13"/>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A69" s="13"/>
+      <c r="B69" s="13"/>
+      <c r="C69" s="13"/>
+    </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="E11:F11"/>
-    <mergeCell ref="B46:E48"/>
+    <mergeCell ref="B48:E50"/>
     <mergeCell ref="F15:F17"/>
   </mergeCells>
   <hyperlinks>
@@ -2409,25 +2406,25 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:O16"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="5.28515625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="8.42578125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="18.5703125" customWidth="1"/>
-    <col min="4" max="4" width="0.140625" hidden="1" customWidth="1"/>
-    <col min="5" max="5" width="13.7109375" customWidth="1"/>
-    <col min="6" max="6" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.42578125" customWidth="1"/>
-    <col min="8" max="8" width="9.28515625" customWidth="1"/>
-    <col min="9" max="9" width="13.140625" hidden="1" customWidth="1"/>
-    <col min="10" max="10" width="17.85546875" customWidth="1"/>
-    <col min="11" max="11" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="14.28515625" customWidth="1"/>
-    <col min="13" max="13" width="13.42578125" customWidth="1"/>
-    <col min="15" max="15" width="11.42578125" style="16"/>
+    <col min="1" max="1" width="5.33203125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="8.44140625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="18.5546875" customWidth="1"/>
+    <col min="4" max="4" width="0.109375" hidden="1" customWidth="1"/>
+    <col min="5" max="5" width="13.6640625" customWidth="1"/>
+    <col min="6" max="6" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.44140625" customWidth="1"/>
+    <col min="8" max="8" width="9.33203125" customWidth="1"/>
+    <col min="9" max="9" width="13.109375" hidden="1" customWidth="1"/>
+    <col min="10" max="10" width="17.88671875" customWidth="1"/>
+    <col min="11" max="11" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="14.33203125" customWidth="1"/>
+    <col min="13" max="13" width="13.44140625" customWidth="1"/>
+    <col min="15" max="15" width="11.44140625" style="16"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A1" s="107" t="s">
         <v>55</v>
       </c>
@@ -2443,16 +2440,16 @@
       <c r="I1" s="109"/>
       <c r="J1" s="109"/>
       <c r="K1" s="112">
-        <f>'detalle y gastos'!C39</f>
-        <v>718194.55</v>
+        <f>'detalle y gastos'!C41</f>
+        <v>1481938.0899999999</v>
       </c>
       <c r="L1" s="112"/>
       <c r="M1" s="113"/>
     </row>
-    <row r="2" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="114" t="str">
         <f>'detalle y gastos'!E7</f>
-        <v>Liquidacion mes de JULIO</v>
+        <v>Liquidacion mes de AGOSTO</v>
       </c>
       <c r="B2" s="56"/>
       <c r="C2" s="56"/>
@@ -2469,7 +2466,7 @@
       <c r="L2" s="90"/>
       <c r="M2" s="115"/>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3" s="29" t="s">
         <v>0</v>
       </c>
@@ -2510,7 +2507,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A4" s="29"/>
       <c r="B4" s="7"/>
       <c r="C4" s="7"/>
@@ -2538,7 +2535,7 @@
       </c>
       <c r="L4" s="51" t="str">
         <f>'detalle y gastos'!F7</f>
-        <v>Vto. 17/08</v>
+        <v>Vto. 17/09</v>
       </c>
       <c r="M4" s="139" t="str">
         <f>O4</f>
@@ -2548,7 +2545,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A5" s="117">
         <v>1</v>
       </c>
@@ -2579,7 +2576,7 @@
       </c>
       <c r="J5" s="27">
         <f>K$1/5</f>
-        <v>143638.91</v>
+        <v>296387.61799999996</v>
       </c>
       <c r="K5" s="93">
         <f>K2*D5</f>
@@ -2587,14 +2584,14 @@
       </c>
       <c r="L5" s="10">
         <f>J5+K5+H5+G5</f>
-        <v>143638.91</v>
+        <v>296387.61799999996</v>
       </c>
       <c r="M5" s="28">
         <f>L5*4%+L5</f>
-        <v>149384.4664</v>
-      </c>
-    </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+        <v>308243.12271999998</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A6" s="117">
         <v>2</v>
       </c>
@@ -2625,7 +2622,7 @@
       </c>
       <c r="J6" s="27">
         <f t="shared" ref="J6:J9" si="1">K$1/5</f>
-        <v>143638.91</v>
+        <v>296387.61799999996</v>
       </c>
       <c r="K6" s="93">
         <f>K2*D6</f>
@@ -2633,14 +2630,14 @@
       </c>
       <c r="L6" s="10">
         <f>J6+K6+H6+G6</f>
-        <v>143638.91</v>
+        <v>296387.61799999996</v>
       </c>
       <c r="M6" s="28">
         <f t="shared" ref="M6:M9" si="2">L6*4%+L6</f>
-        <v>149384.4664</v>
-      </c>
-    </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+        <v>308243.12271999998</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A7" s="117">
         <v>3</v>
       </c>
@@ -2671,7 +2668,7 @@
       </c>
       <c r="J7" s="27">
         <f t="shared" si="1"/>
-        <v>143638.91</v>
+        <v>296387.61799999996</v>
       </c>
       <c r="K7" s="93">
         <f>K2*D7</f>
@@ -2679,14 +2676,14 @@
       </c>
       <c r="L7" s="10">
         <f>J7+K7+H7+G7</f>
-        <v>143638.91</v>
+        <v>296387.61799999996</v>
       </c>
       <c r="M7" s="28">
         <f t="shared" si="2"/>
-        <v>149384.4664</v>
-      </c>
-    </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+        <v>308243.12271999998</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8" s="117">
         <v>4</v>
       </c>
@@ -2716,7 +2713,7 @@
       </c>
       <c r="J8" s="27">
         <f t="shared" si="1"/>
-        <v>143638.91</v>
+        <v>296387.61799999996</v>
       </c>
       <c r="K8" s="93">
         <f>K2*D8</f>
@@ -2724,14 +2721,14 @@
       </c>
       <c r="L8" s="10">
         <f>J8+K8+H8+G8</f>
-        <v>137893.86742400003</v>
+        <v>290642.57542399998</v>
       </c>
       <c r="M8" s="28">
         <f t="shared" si="2"/>
-        <v>143409.62212096003</v>
-      </c>
-    </row>
-    <row r="9" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>302268.27844095998</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="118">
         <v>5</v>
       </c>
@@ -2761,7 +2758,7 @@
       </c>
       <c r="J9" s="127">
         <f t="shared" si="1"/>
-        <v>143638.91</v>
+        <v>296387.61799999996</v>
       </c>
       <c r="K9" s="128">
         <f>K2*D9</f>
@@ -2769,14 +2766,14 @@
       </c>
       <c r="L9" s="126">
         <f>J9+K9+H9+G9</f>
-        <v>184816.0564</v>
+        <v>337564.76439999999</v>
       </c>
       <c r="M9" s="129">
         <f t="shared" si="2"/>
-        <v>192208.69865599999</v>
-      </c>
-    </row>
-    <row r="10" spans="1:15" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+        <v>351067.35497599997</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="130" t="s">
         <v>8</v>
       </c>
@@ -2808,7 +2805,7 @@
       </c>
       <c r="J10" s="137">
         <f t="shared" si="4"/>
-        <v>718194.55</v>
+        <v>1481938.0899999999</v>
       </c>
       <c r="K10" s="136">
         <f t="shared" si="4"/>
@@ -2816,14 +2813,14 @@
       </c>
       <c r="L10" s="135">
         <f t="shared" si="4"/>
-        <v>753626.65382400004</v>
+        <v>1517370.1938239997</v>
       </c>
       <c r="M10" s="135">
         <f t="shared" si="4"/>
-        <v>783771.71997695998</v>
-      </c>
-    </row>
-    <row r="11" spans="1:15" ht="51.75" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+        <v>1578065.0015769599</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" ht="51.75" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="144"/>
       <c r="B11" s="144"/>
       <c r="C11" s="144"/>
@@ -2838,10 +2835,10 @@
       <c r="L11" s="144"/>
       <c r="M11" s="144"/>
     </row>
-    <row r="12" spans="1:15" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:15" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="M12" s="6"/>
     </row>
-    <row r="13" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="C13" s="145"/>
       <c r="D13" s="145"/>
       <c r="E13" s="145"/>
@@ -2853,7 +2850,7 @@
       <c r="K13" s="145"/>
       <c r="L13" s="145"/>
     </row>
-    <row r="14" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="C14" s="145"/>
       <c r="D14" s="145"/>
       <c r="E14" s="145"/>
@@ -2865,7 +2862,7 @@
       <c r="K14" s="145"/>
       <c r="L14" s="145"/>
     </row>
-    <row r="15" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="C15" s="145"/>
       <c r="D15" s="145"/>
       <c r="E15" s="145"/>
@@ -2877,7 +2874,7 @@
       <c r="K15" s="145"/>
       <c r="L15" s="145"/>
     </row>
-    <row r="16" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="C16" s="145"/>
       <c r="D16" s="145"/>
       <c r="E16" s="145"/>
@@ -2903,12 +2900,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:G12"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="3" width="13.140625" customWidth="1"/>
+    <col min="3" max="3" width="13.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="151" t="s">
         <v>24</v>
       </c>
@@ -2919,7 +2916,7 @@
       <c r="F1" s="70"/>
       <c r="G1" s="70"/>
     </row>
-    <row r="2" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="154" t="s">
         <v>50</v>
       </c>
@@ -2932,7 +2929,7 @@
       <c r="F2" s="71"/>
       <c r="G2" s="71"/>
     </row>
-    <row r="3" spans="1:7" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A3" s="159" t="s">
         <v>0</v>
       </c>
@@ -2955,7 +2952,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="160"/>
       <c r="B4" s="160"/>
       <c r="C4" s="160"/>
@@ -2964,7 +2961,7 @@
       <c r="F4" s="147"/>
       <c r="G4" s="147"/>
     </row>
-    <row r="5" spans="1:7" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="72">
         <v>1</v>
       </c>
@@ -2987,7 +2984,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="72">
         <v>2</v>
       </c>
@@ -3010,7 +3007,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="72">
         <v>3</v>
       </c>
@@ -3033,7 +3030,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="72">
         <v>4</v>
       </c>
@@ -3056,7 +3053,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="72">
         <v>5</v>
       </c>
@@ -3079,7 +3076,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="77">
         <v>6</v>
       </c>
@@ -3102,7 +3099,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="82" t="s">
         <v>8</v>
       </c>
@@ -3121,7 +3118,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="148"/>
       <c r="B12" s="149"/>
       <c r="C12" s="149"/>

</xml_diff>